<commit_message>
finalizo excel p4 medioambiente
</commit_message>
<xml_diff>
--- a/medioambiente/practica4medioambiente.xlsx
+++ b/medioambiente/practica4medioambiente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andres\Practicas-Fisica\medioambiente\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF9D6FB-AF05-4E6C-8241-6E0E29E6340B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6472CA9-D1F4-49E6-8588-B076671C38FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{310D8BF0-0524-4B4E-8AE5-C888D12EF181}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>dBA</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>dBC  ruido</t>
+  </si>
+  <si>
+    <t>movil dbA</t>
   </si>
 </sst>
 </file>
@@ -425,10 +428,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CEF571A-872F-475B-B43F-76A4D3C23FE6}">
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -444,8 +447,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -461,8 +467,11 @@
       <c r="E2">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>(ROW()-2)*10</f>
         <v>10</v>
@@ -479,8 +488,11 @@
       <c r="E3">
         <v>55.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" ref="A4:A61" si="0">(ROW()-2)*10</f>
         <v>20</v>
@@ -497,8 +509,11 @@
       <c r="E4">
         <v>55.6</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -515,8 +530,11 @@
       <c r="E5">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G5">
+        <v>72.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -533,8 +551,11 @@
       <c r="E6">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G6">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -551,8 +572,11 @@
       <c r="E7">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -569,8 +593,11 @@
       <c r="E8">
         <v>55.1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <v>73.099999999999994</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>70</v>
@@ -587,8 +614,11 @@
       <c r="E9">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -605,8 +635,11 @@
       <c r="E10">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <v>75.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>90</v>
@@ -623,8 +656,11 @@
       <c r="E11">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <v>72.900000000000006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>100</v>
@@ -641,8 +677,11 @@
       <c r="E12">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>110</v>
@@ -659,8 +698,11 @@
       <c r="E13">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>120</v>
@@ -677,8 +719,11 @@
       <c r="E14">
         <v>56.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G14">
+        <v>72.099999999999994</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>130</v>
@@ -695,8 +740,11 @@
       <c r="E15">
         <v>55.9</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G15">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>140</v>
@@ -713,8 +761,11 @@
       <c r="E16">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G16">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>150</v>
@@ -731,8 +782,11 @@
       <c r="E17">
         <v>56.1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G17">
+        <v>74.599999999999994</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>160</v>
@@ -749,8 +803,11 @@
       <c r="E18">
         <v>56.3</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G18">
+        <v>74.900000000000006</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>170</v>
@@ -767,8 +824,11 @@
       <c r="E19">
         <v>56.4</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G19">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>180</v>
@@ -785,8 +845,11 @@
       <c r="E20">
         <v>56.6</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G20">
+        <v>73.599999999999994</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>190</v>
@@ -803,8 +866,11 @@
       <c r="E21">
         <v>56.8</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G21">
+        <v>74.599999999999994</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>200</v>
@@ -821,8 +887,11 @@
       <c r="E22">
         <v>56.9</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G22">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>210</v>
@@ -839,8 +908,11 @@
       <c r="E23">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G23">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>220</v>
@@ -857,8 +929,11 @@
       <c r="E24">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G24">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>230</v>
@@ -875,8 +950,11 @@
       <c r="E25">
         <v>56</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G25">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>240</v>
@@ -893,8 +971,11 @@
       <c r="E26">
         <v>56.4</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G26">
+        <v>74.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>250</v>
@@ -911,8 +992,11 @@
       <c r="E27">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G27">
+        <v>73.599999999999994</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>260</v>
@@ -929,8 +1013,11 @@
       <c r="E28">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G28">
+        <v>74.400000000000006</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>270</v>
@@ -947,8 +1034,11 @@
       <c r="E29">
         <v>56</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G29">
+        <v>72.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>280</v>
@@ -965,8 +1055,11 @@
       <c r="E30">
         <v>56.5</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G30">
+        <v>73.599999999999994</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>290</v>
@@ -983,8 +1076,11 @@
       <c r="E31">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G31">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>300</v>
@@ -1001,8 +1097,11 @@
       <c r="E32">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G32">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>310</v>
@@ -1019,8 +1118,11 @@
       <c r="E33">
         <v>55.7</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G33">
+        <v>73.900000000000006</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>320</v>
@@ -1037,8 +1139,11 @@
       <c r="E34">
         <v>55.9</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G34">
+        <v>72.099999999999994</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <f t="shared" si="0"/>
         <v>330</v>
@@ -1055,8 +1160,11 @@
       <c r="E35">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G35">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>340</v>
@@ -1073,8 +1181,11 @@
       <c r="E36">
         <v>56.1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G36">
+        <v>74.900000000000006</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>350</v>
@@ -1091,8 +1202,11 @@
       <c r="E37">
         <v>56</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G37">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <f t="shared" si="0"/>
         <v>360</v>
@@ -1109,8 +1223,11 @@
       <c r="E38">
         <v>55.9</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G38">
+        <v>73.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <f t="shared" si="0"/>
         <v>370</v>
@@ -1127,8 +1244,11 @@
       <c r="E39">
         <v>55.6</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G39">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>380</v>
@@ -1145,8 +1265,11 @@
       <c r="E40">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G40">
+        <v>73.099999999999994</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>390</v>
@@ -1163,8 +1286,11 @@
       <c r="E41">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G41">
+        <v>73.900000000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>400</v>
@@ -1181,8 +1307,11 @@
       <c r="E42">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G42">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>410</v>
@@ -1199,8 +1328,11 @@
       <c r="E43">
         <v>55.5</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G43">
+        <v>75.2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>420</v>
@@ -1217,8 +1349,11 @@
       <c r="E44">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G44">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>430</v>
@@ -1235,8 +1370,11 @@
       <c r="E45">
         <v>55.2</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G45">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>440</v>
@@ -1253,8 +1391,11 @@
       <c r="E46">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G46">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>450</v>
@@ -1271,8 +1412,11 @@
       <c r="E47">
         <v>55.6</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G47">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>460</v>
@@ -1289,8 +1433,11 @@
       <c r="E48">
         <v>56.8</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G48">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <f t="shared" si="0"/>
         <v>470</v>
@@ -1307,8 +1454,11 @@
       <c r="E49">
         <v>56.6</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G49">
+        <v>74.400000000000006</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <f t="shared" si="0"/>
         <v>480</v>
@@ -1325,8 +1475,11 @@
       <c r="E50">
         <v>56.4</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G50">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <f t="shared" si="0"/>
         <v>490</v>
@@ -1343,8 +1496,11 @@
       <c r="E51">
         <v>56.2</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G51">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <f t="shared" si="0"/>
         <v>500</v>
@@ -1361,8 +1517,11 @@
       <c r="E52">
         <v>56</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G52">
+        <v>74.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <f t="shared" si="0"/>
         <v>510</v>
@@ -1379,8 +1538,11 @@
       <c r="E53">
         <v>55.5</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G53">
+        <v>73.099999999999994</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <f t="shared" si="0"/>
         <v>520</v>
@@ -1397,8 +1559,11 @@
       <c r="E54">
         <v>55</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G54">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <f t="shared" si="0"/>
         <v>530</v>
@@ -1415,8 +1580,11 @@
       <c r="E55">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G55">
+        <v>74.599999999999994</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56">
         <f t="shared" si="0"/>
         <v>540</v>
@@ -1433,8 +1601,11 @@
       <c r="E56">
         <v>55.6</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G56">
+        <v>72.900000000000006</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57">
         <f t="shared" si="0"/>
         <v>550</v>
@@ -1451,8 +1622,11 @@
       <c r="E57">
         <v>56.2</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G57">
+        <v>72.599999999999994</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <f t="shared" si="0"/>
         <v>560</v>
@@ -1469,8 +1643,11 @@
       <c r="E58">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G58">
+        <v>74.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <f t="shared" si="0"/>
         <v>570</v>
@@ -1487,8 +1664,11 @@
       <c r="E59">
         <v>55.4</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G59">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <f t="shared" si="0"/>
         <v>580</v>
@@ -1505,8 +1685,11 @@
       <c r="E60">
         <v>55.6</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G60">
+        <v>73.599999999999994</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61">
         <f t="shared" si="0"/>
         <v>590</v>
@@ -1523,8 +1706,11 @@
       <c r="E61">
         <v>55.3</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G61">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>600</v>
       </c>
@@ -1539,6 +1725,9 @@
       </c>
       <c r="E62">
         <v>55.8</v>
+      </c>
+      <c r="G62">
+        <v>74.599999999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>